<commit_message>
feat: optional soul manufacture and attack-move interrupt distance gate (v0.75.35)
Soul slot optional with Soul_00/Class_Servants defaults; SetMoving only force-cuts Attack when move target XZ distance exceeds 0.4.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/制造_灵魂配置表_Manufacture_SoulConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/制造_灵魂配置表_Manufacture_SoulConfig.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="80">
   <si>
     <t>灵魂ID</t>
   </si>
@@ -106,22 +106,28 @@
     <t>ControlPowerCost</t>
   </si>
   <si>
+    <t>Soul_00</t>
+  </si>
+  <si>
+    <t>Class_Servants</t>
+  </si>
+  <si>
+    <t>Melee</t>
+  </si>
+  <si>
+    <t>Nearest</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
     <t>Soul_01</t>
   </si>
   <si>
     <t>Class_Warrior</t>
   </si>
   <si>
-    <t>Melee</t>
-  </si>
-  <si>
     <t/>
-  </si>
-  <si>
-    <t>Nearest</t>
-  </si>
-  <si>
-    <t>Normal</t>
   </si>
   <si>
     <t>10</t>
@@ -278,14 +284,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -747,148 +746,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1241,7 +1240,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
     <col min="2" max="2" width="16.125" customWidth="1"/>
@@ -1337,254 +1336,277 @@
       <c r="C4" t="s">
         <v>26</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>27</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>28</v>
       </c>
-      <c r="F4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" t="s">
-        <v>31</v>
+      <c r="G4">
+        <v>5</v>
+      </c>
+      <c r="H4">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" t="s">
+      <c r="H5" t="s">
         <v>33</v>
-      </c>
-      <c r="C5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" t="s">
         <v>40</v>
       </c>
-      <c r="B6" t="s">
+      <c r="H6" t="s">
         <v>41</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E6" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" t="s">
-        <v>44</v>
-      </c>
-      <c r="G6" t="s">
-        <v>45</v>
-      </c>
-      <c r="H6" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" t="s">
         <v>47</v>
       </c>
-      <c r="B7" t="s">
+      <c r="H7" t="s">
         <v>48</v>
-      </c>
-      <c r="C7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G7" t="s">
-        <v>49</v>
-      </c>
-      <c r="H7" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
         <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="G8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" t="s">
         <v>56</v>
       </c>
-      <c r="B9" t="s">
+      <c r="H9" t="s">
         <v>57</v>
-      </c>
-      <c r="C9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" t="s">
-        <v>58</v>
-      </c>
-      <c r="E9" t="s">
-        <v>43</v>
-      </c>
-      <c r="F9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G9" t="s">
-        <v>59</v>
-      </c>
-      <c r="H9" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
         <v>60</v>
       </c>
-      <c r="B10" t="s">
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" t="s">
+        <v>46</v>
+      </c>
+      <c r="G10" t="s">
         <v>61</v>
       </c>
-      <c r="C10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" t="s">
-        <v>28</v>
-      </c>
-      <c r="F10" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" t="s">
-        <v>62</v>
-      </c>
       <c r="H10" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" t="s">
         <v>64</v>
       </c>
-      <c r="B11" t="s">
+      <c r="H11" t="s">
         <v>65</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E11" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11" t="s">
-        <v>37</v>
-      </c>
-      <c r="G11" t="s">
-        <v>67</v>
-      </c>
-      <c r="H11" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" t="s">
         <v>69</v>
       </c>
-      <c r="B12" t="s">
+      <c r="H12" t="s">
         <v>70</v>
-      </c>
-      <c r="C12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D12" t="s">
-        <v>71</v>
-      </c>
-      <c r="E12" t="s">
-        <v>43</v>
-      </c>
-      <c r="F12" t="s">
-        <v>44</v>
-      </c>
-      <c r="G12" t="s">
-        <v>72</v>
-      </c>
-      <c r="H12" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" t="s">
         <v>74</v>
       </c>
-      <c r="B13" t="s">
+      <c r="H13" t="s">
         <v>75</v>
       </c>
-      <c r="C13" t="s">
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" t="s">
         <v>26</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" t="s">
         <v>27</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F14" t="s">
         <v>28</v>
       </c>
-      <c r="F13" t="s">
-        <v>29</v>
-      </c>
-      <c r="G13" t="s">
-        <v>76</v>
-      </c>
-      <c r="H13" t="s">
-        <v>77</v>
+      <c r="G14" t="s">
+        <v>78</v>
+      </c>
+      <c r="H14" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>